<commit_message>
New style for figures looking like GraphPad Prism
</commit_message>
<xml_diff>
--- a/data/viability.xlsx
+++ b/data/viability.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Depalma-Lab/Alexia/3.Experiments/20251028-Thawing_Dcp_test/ThawingDCPs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Depalma-Lab/Alexia/5.Figures_python/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6458A1C6-795B-EB4A-B9D2-6DFA4B9FD583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D4D9E53-427B-F247-B1EE-9B8B93072B14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8340" yWindow="740" windowWidth="21060" windowHeight="17000" activeTab="5" xr2:uid="{04F21ADD-521C-3D43-8BD2-2F70976D6201}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" activeTab="6" xr2:uid="{04F21ADD-521C-3D43-8BD2-2F70976D6201}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Flow-csv" sheetId="4" r:id="rId4"/>
     <sheet name="Viability " sheetId="5" r:id="rId5"/>
     <sheet name="Feuil3" sheetId="6" r:id="rId6"/>
+    <sheet name="Feuil4" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="685" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="55">
   <si>
     <t>Before thawing</t>
   </si>
@@ -10809,6 +10810,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5" customWidth="1"/>
+    <col min="4" max="4" width="23.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:15" x14ac:dyDescent="0.2">
@@ -12212,4 +12214,1099 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74EEED9E-8C0E-5D44-935C-575B058CDDAA}">
+  <dimension ref="B2:E80"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6">
+        <v>225000</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E7">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8">
+        <v>160000</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10">
+        <v>305000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12">
+        <v>465000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14">
+        <v>670000</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17">
+        <v>105000</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>42</v>
+      </c>
+      <c r="D19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" t="s">
+        <v>19</v>
+      </c>
+      <c r="E20">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" t="s">
+        <v>19</v>
+      </c>
+      <c r="E21">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>19</v>
+      </c>
+      <c r="E22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>42</v>
+      </c>
+      <c r="D23" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" t="s">
+        <v>19</v>
+      </c>
+      <c r="E24">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25">
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>42</v>
+      </c>
+      <c r="D27" t="s">
+        <v>19</v>
+      </c>
+      <c r="E27">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" t="s">
+        <v>19</v>
+      </c>
+      <c r="E28">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>2</v>
+      </c>
+      <c r="C30" t="s">
+        <v>42</v>
+      </c>
+      <c r="D30" t="s">
+        <v>47</v>
+      </c>
+      <c r="E30">
+        <v>135000</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>2</v>
+      </c>
+      <c r="C31" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" t="s">
+        <v>47</v>
+      </c>
+      <c r="E31">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>42</v>
+      </c>
+      <c r="D32" t="s">
+        <v>47</v>
+      </c>
+      <c r="E32">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>42</v>
+      </c>
+      <c r="D34" t="s">
+        <v>47</v>
+      </c>
+      <c r="E34">
+        <v>220000</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" t="s">
+        <v>47</v>
+      </c>
+      <c r="E35">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>5</v>
+      </c>
+      <c r="C36" t="s">
+        <v>42</v>
+      </c>
+      <c r="D36" t="s">
+        <v>47</v>
+      </c>
+      <c r="E36">
+        <v>175000</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>5</v>
+      </c>
+      <c r="C37" t="s">
+        <v>43</v>
+      </c>
+      <c r="D37" t="s">
+        <v>47</v>
+      </c>
+      <c r="E37">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" t="s">
+        <v>42</v>
+      </c>
+      <c r="D38" t="s">
+        <v>47</v>
+      </c>
+      <c r="E38">
+        <v>290000</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>6</v>
+      </c>
+      <c r="C39" t="s">
+        <v>43</v>
+      </c>
+      <c r="D39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E39">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" t="s">
+        <v>42</v>
+      </c>
+      <c r="D40" t="s">
+        <v>47</v>
+      </c>
+      <c r="E40">
+        <v>260000</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" t="s">
+        <v>43</v>
+      </c>
+      <c r="D41" t="s">
+        <v>47</v>
+      </c>
+      <c r="E41">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>1</v>
+      </c>
+      <c r="D42" t="s">
+        <v>48</v>
+      </c>
+      <c r="E42">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>2</v>
+      </c>
+      <c r="C43" t="s">
+        <v>42</v>
+      </c>
+      <c r="D43" t="s">
+        <v>48</v>
+      </c>
+      <c r="E43">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>2</v>
+      </c>
+      <c r="C44" t="s">
+        <v>43</v>
+      </c>
+      <c r="D44" t="s">
+        <v>48</v>
+      </c>
+      <c r="E44">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" t="s">
+        <v>48</v>
+      </c>
+      <c r="E45">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>43</v>
+      </c>
+      <c r="D46" t="s">
+        <v>48</v>
+      </c>
+      <c r="E46">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B47" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>42</v>
+      </c>
+      <c r="D47" t="s">
+        <v>48</v>
+      </c>
+      <c r="E47">
+        <v>230000</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" t="s">
+        <v>43</v>
+      </c>
+      <c r="D48" t="s">
+        <v>48</v>
+      </c>
+      <c r="E48">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B49" t="s">
+        <v>5</v>
+      </c>
+      <c r="C49" t="s">
+        <v>42</v>
+      </c>
+      <c r="D49" t="s">
+        <v>48</v>
+      </c>
+      <c r="E49">
+        <v>490000</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B50" t="s">
+        <v>5</v>
+      </c>
+      <c r="C50" t="s">
+        <v>43</v>
+      </c>
+      <c r="D50" t="s">
+        <v>48</v>
+      </c>
+      <c r="E50">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B51" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" t="s">
+        <v>42</v>
+      </c>
+      <c r="D51" t="s">
+        <v>48</v>
+      </c>
+      <c r="E51">
+        <v>735000</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B52" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" t="s">
+        <v>43</v>
+      </c>
+      <c r="D52" t="s">
+        <v>48</v>
+      </c>
+      <c r="E52">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B53" t="s">
+        <v>7</v>
+      </c>
+      <c r="C53" t="s">
+        <v>42</v>
+      </c>
+      <c r="D53" t="s">
+        <v>48</v>
+      </c>
+      <c r="E53">
+        <v>1255000</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B54" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" t="s">
+        <v>43</v>
+      </c>
+      <c r="D54" t="s">
+        <v>48</v>
+      </c>
+      <c r="E54">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B55" t="s">
+        <v>1</v>
+      </c>
+      <c r="D55" t="s">
+        <v>17</v>
+      </c>
+      <c r="E55">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B56" t="s">
+        <v>2</v>
+      </c>
+      <c r="C56" t="s">
+        <v>42</v>
+      </c>
+      <c r="D56" t="s">
+        <v>17</v>
+      </c>
+      <c r="E56">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
+        <v>2</v>
+      </c>
+      <c r="C57" t="s">
+        <v>43</v>
+      </c>
+      <c r="D57" t="s">
+        <v>17</v>
+      </c>
+      <c r="E57">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B58" t="s">
+        <v>3</v>
+      </c>
+      <c r="C58" t="s">
+        <v>42</v>
+      </c>
+      <c r="D58" t="s">
+        <v>17</v>
+      </c>
+      <c r="E58">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B59" t="s">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>43</v>
+      </c>
+      <c r="D59" t="s">
+        <v>17</v>
+      </c>
+      <c r="E59">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B60" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" t="s">
+        <v>42</v>
+      </c>
+      <c r="D60" t="s">
+        <v>17</v>
+      </c>
+      <c r="E60">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B61" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" t="s">
+        <v>43</v>
+      </c>
+      <c r="D61" t="s">
+        <v>17</v>
+      </c>
+      <c r="E61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B62" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62" t="s">
+        <v>42</v>
+      </c>
+      <c r="D62" t="s">
+        <v>17</v>
+      </c>
+      <c r="E62">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B63" t="s">
+        <v>5</v>
+      </c>
+      <c r="C63" t="s">
+        <v>43</v>
+      </c>
+      <c r="D63" t="s">
+        <v>17</v>
+      </c>
+      <c r="E63">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B64" t="s">
+        <v>6</v>
+      </c>
+      <c r="C64" t="s">
+        <v>42</v>
+      </c>
+      <c r="D64" t="s">
+        <v>17</v>
+      </c>
+      <c r="E64">
+        <v>65000</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B65" t="s">
+        <v>6</v>
+      </c>
+      <c r="C65" t="s">
+        <v>43</v>
+      </c>
+      <c r="D65" t="s">
+        <v>17</v>
+      </c>
+      <c r="E65">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B66" t="s">
+        <v>7</v>
+      </c>
+      <c r="C66" t="s">
+        <v>42</v>
+      </c>
+      <c r="D66" t="s">
+        <v>17</v>
+      </c>
+      <c r="E66">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B67" t="s">
+        <v>7</v>
+      </c>
+      <c r="C67" t="s">
+        <v>43</v>
+      </c>
+      <c r="D67" t="s">
+        <v>17</v>
+      </c>
+      <c r="E67">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="68" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B68" t="s">
+        <v>1</v>
+      </c>
+      <c r="D68" t="s">
+        <v>46</v>
+      </c>
+      <c r="E68">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="69" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B69" t="s">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>42</v>
+      </c>
+      <c r="D69" t="s">
+        <v>46</v>
+      </c>
+      <c r="E69">
+        <v>55000</v>
+      </c>
+    </row>
+    <row r="70" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B70" t="s">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>43</v>
+      </c>
+      <c r="D70" t="s">
+        <v>46</v>
+      </c>
+      <c r="E70">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="71" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B71" t="s">
+        <v>3</v>
+      </c>
+      <c r="C71" t="s">
+        <v>42</v>
+      </c>
+      <c r="D71" t="s">
+        <v>46</v>
+      </c>
+      <c r="E71">
+        <v>95000</v>
+      </c>
+    </row>
+    <row r="72" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B72" t="s">
+        <v>3</v>
+      </c>
+      <c r="C72" t="s">
+        <v>43</v>
+      </c>
+      <c r="D72" t="s">
+        <v>46</v>
+      </c>
+      <c r="E72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B73" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" t="s">
+        <v>42</v>
+      </c>
+      <c r="D73" t="s">
+        <v>46</v>
+      </c>
+      <c r="E73">
+        <v>185000</v>
+      </c>
+    </row>
+    <row r="74" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B74" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" t="s">
+        <v>43</v>
+      </c>
+      <c r="D74" t="s">
+        <v>46</v>
+      </c>
+      <c r="E74">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="75" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B75" t="s">
+        <v>5</v>
+      </c>
+      <c r="C75" t="s">
+        <v>42</v>
+      </c>
+      <c r="D75" t="s">
+        <v>46</v>
+      </c>
+      <c r="E75">
+        <v>455000</v>
+      </c>
+    </row>
+    <row r="76" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B76" t="s">
+        <v>5</v>
+      </c>
+      <c r="C76" t="s">
+        <v>43</v>
+      </c>
+      <c r="D76" t="s">
+        <v>46</v>
+      </c>
+      <c r="E76">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="77" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B77" t="s">
+        <v>6</v>
+      </c>
+      <c r="C77" t="s">
+        <v>42</v>
+      </c>
+      <c r="D77" t="s">
+        <v>46</v>
+      </c>
+      <c r="E77">
+        <v>280000</v>
+      </c>
+    </row>
+    <row r="78" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B78" t="s">
+        <v>6</v>
+      </c>
+      <c r="C78" t="s">
+        <v>43</v>
+      </c>
+      <c r="D78" t="s">
+        <v>46</v>
+      </c>
+      <c r="E78">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="79" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B79" t="s">
+        <v>7</v>
+      </c>
+      <c r="C79" t="s">
+        <v>42</v>
+      </c>
+      <c r="D79" t="s">
+        <v>46</v>
+      </c>
+      <c r="E79">
+        <v>650000</v>
+      </c>
+    </row>
+    <row r="80" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B80" t="s">
+        <v>7</v>
+      </c>
+      <c r="C80" t="s">
+        <v>43</v>
+      </c>
+      <c r="D80" t="s">
+        <v>46</v>
+      </c>
+      <c r="E80">
+        <v>20000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>